<commit_message>
Adiciona colunas pontuacao_a e pontuacao_b separadas para discursivas
</commit_message>
<xml_diff>
--- a/questoes_oab_2fase.xlsx
+++ b/questoes_oab_2fase.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prova OAB 2a Fase" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prova OAB 2a Fase'!$A$1:$H$192</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prova OAB 2a Fase'!$A$1:$J$192</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:J192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -511,7 +511,9 @@
     <col width="70" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
-    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -551,6 +553,16 @@
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Pontuacao A</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Pontuacao B</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Distribuicao de Pontos</t>
         </is>
@@ -569,6 +581,8 @@
       <c r="F2" s="3" t="n"/>
       <c r="G2" s="3" t="n"/>
       <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -607,6 +621,8 @@
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr"/>
+      <c r="J3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -645,6 +661,8 @@
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr"/>
+      <c r="I4" s="5" t="inlineStr"/>
+      <c r="J4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -683,6 +701,8 @@
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -721,6 +741,8 @@
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr"/>
+      <c r="I6" s="5" t="inlineStr"/>
+      <c r="J6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -760,6 +782,8 @@
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -802,6 +826,8 @@
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr"/>
+      <c r="I8" s="5" t="inlineStr"/>
+      <c r="J8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -844,6 +870,8 @@
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr"/>
+      <c r="J9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -885,6 +913,8 @@
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr"/>
+      <c r="I10" s="5" t="inlineStr"/>
+      <c r="J10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -923,6 +953,8 @@
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -961,6 +993,8 @@
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr"/>
+      <c r="I12" s="5" t="inlineStr"/>
+      <c r="J12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -999,6 +1033,8 @@
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr"/>
+      <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1043,6 +1079,8 @@
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr"/>
+      <c r="I14" s="5" t="inlineStr"/>
+      <c r="J14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1086,6 +1124,8 @@
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr"/>
+      <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1128,6 +1168,8 @@
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr"/>
+      <c r="I16" s="5" t="inlineStr"/>
+      <c r="J16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1169,6 +1211,8 @@
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr"/>
+      <c r="I17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1211,6 +1255,8 @@
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr"/>
+      <c r="I18" s="5" t="inlineStr"/>
+      <c r="J18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1249,6 +1295,8 @@
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr"/>
+      <c r="I19" s="4" t="inlineStr"/>
+      <c r="J19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1290,6 +1338,8 @@
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr"/>
+      <c r="I20" s="5" t="inlineStr"/>
+      <c r="J20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1328,6 +1378,8 @@
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr"/>
+      <c r="I21" s="4" t="inlineStr"/>
+      <c r="J21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -1365,6 +1417,8 @@
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr"/>
+      <c r="I22" s="5" t="inlineStr"/>
+      <c r="J22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1404,6 +1458,8 @@
       </c>
       <c r="G23" s="4" t="inlineStr"/>
       <c r="H23" s="4" t="inlineStr"/>
+      <c r="I23" s="4" t="inlineStr"/>
+      <c r="J23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -1447,6 +1503,8 @@
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr"/>
+      <c r="I24" s="5" t="inlineStr"/>
+      <c r="J24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1489,6 +1547,8 @@
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
+      <c r="I25" s="4" t="inlineStr"/>
+      <c r="J25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -1530,6 +1590,8 @@
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr"/>
+      <c r="I26" s="5" t="inlineStr"/>
+      <c r="J26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1572,6 +1634,8 @@
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
+      <c r="I27" s="4" t="inlineStr"/>
+      <c r="J27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -1614,6 +1678,8 @@
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr"/>
+      <c r="I28" s="5" t="inlineStr"/>
+      <c r="J28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1656,6 +1722,8 @@
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
+      <c r="I29" s="4" t="inlineStr"/>
+      <c r="J29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -1699,6 +1767,8 @@
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr"/>
+      <c r="I30" s="5" t="inlineStr"/>
+      <c r="J30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1738,6 +1808,8 @@
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
+      <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -1780,6 +1852,8 @@
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr"/>
+      <c r="I32" s="5" t="inlineStr"/>
+      <c r="J32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -1823,6 +1897,8 @@
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
+      <c r="I33" s="4" t="inlineStr"/>
+      <c r="J33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -1862,6 +1938,8 @@
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr"/>
+      <c r="I34" s="5" t="inlineStr"/>
+      <c r="J34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -1905,6 +1983,8 @@
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
+      <c r="I35" s="4" t="inlineStr"/>
+      <c r="J35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -1947,6 +2027,8 @@
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr"/>
+      <c r="I36" s="5" t="inlineStr"/>
+      <c r="J36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -1989,6 +2071,8 @@
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
+      <c r="I37" s="4" t="inlineStr"/>
+      <c r="J37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -2031,6 +2115,8 @@
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr"/>
+      <c r="I38" s="5" t="inlineStr"/>
+      <c r="J38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -2070,6 +2156,8 @@
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
+      <c r="I39" s="4" t="inlineStr"/>
+      <c r="J39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -2112,6 +2200,8 @@
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr"/>
+      <c r="I40" s="5" t="inlineStr"/>
+      <c r="J40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -2155,6 +2245,8 @@
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
+      <c r="I41" s="4" t="inlineStr"/>
+      <c r="J41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -2196,6 +2288,8 @@
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr"/>
+      <c r="I42" s="5" t="inlineStr"/>
+      <c r="J42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -2234,6 +2328,8 @@
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
+      <c r="I43" s="4" t="inlineStr"/>
+      <c r="J43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -2276,6 +2372,8 @@
         </is>
       </c>
       <c r="H44" s="5" t="inlineStr"/>
+      <c r="I44" s="5" t="inlineStr"/>
+      <c r="J44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -2318,6 +2416,8 @@
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
+      <c r="I45" s="4" t="inlineStr"/>
+      <c r="J45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
@@ -2359,6 +2459,8 @@
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr"/>
+      <c r="I46" s="5" t="inlineStr"/>
+      <c r="J46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -2403,6 +2505,8 @@
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr"/>
+      <c r="I47" s="4" t="inlineStr"/>
+      <c r="J47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
@@ -2446,6 +2550,8 @@
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr"/>
+      <c r="I48" s="5" t="inlineStr"/>
+      <c r="J48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -2490,6 +2596,8 @@
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr"/>
+      <c r="I49" s="4" t="inlineStr"/>
+      <c r="J49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
@@ -2535,6 +2643,8 @@
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr"/>
+      <c r="I50" s="5" t="inlineStr"/>
+      <c r="J50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -2579,6 +2689,8 @@
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr"/>
+      <c r="I51" s="4" t="inlineStr"/>
+      <c r="J51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
@@ -2621,6 +2733,8 @@
         </is>
       </c>
       <c r="H52" s="5" t="inlineStr"/>
+      <c r="I52" s="5" t="inlineStr"/>
+      <c r="J52" s="5" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -2663,6 +2777,8 @@
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr"/>
+      <c r="I53" s="4" t="inlineStr"/>
+      <c r="J53" s="4" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
@@ -2704,6 +2820,8 @@
         </is>
       </c>
       <c r="H54" s="5" t="inlineStr"/>
+      <c r="I54" s="5" t="inlineStr"/>
+      <c r="J54" s="5" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -2741,6 +2859,8 @@
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr"/>
+      <c r="I55" s="4" t="inlineStr"/>
+      <c r="J55" s="4" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
@@ -2784,6 +2904,8 @@
         </is>
       </c>
       <c r="H56" s="5" t="inlineStr"/>
+      <c r="I56" s="5" t="inlineStr"/>
+      <c r="J56" s="5" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -2825,6 +2947,8 @@
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr"/>
+      <c r="I57" s="4" t="inlineStr"/>
+      <c r="J57" s="4" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
@@ -2868,6 +2992,8 @@
         </is>
       </c>
       <c r="H58" s="5" t="inlineStr"/>
+      <c r="I58" s="5" t="inlineStr"/>
+      <c r="J58" s="5" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -2907,6 +3033,8 @@
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr"/>
+      <c r="I59" s="4" t="inlineStr"/>
+      <c r="J59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
@@ -2950,6 +3078,8 @@
         </is>
       </c>
       <c r="H60" s="5" t="inlineStr"/>
+      <c r="I60" s="5" t="inlineStr"/>
+      <c r="J60" s="5" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -2993,6 +3123,8 @@
         </is>
       </c>
       <c r="H61" s="4" t="inlineStr"/>
+      <c r="I61" s="4" t="inlineStr"/>
+      <c r="J61" s="4" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
@@ -3036,6 +3168,8 @@
         </is>
       </c>
       <c r="H62" s="5" t="inlineStr"/>
+      <c r="I62" s="5" t="inlineStr"/>
+      <c r="J62" s="5" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -3078,6 +3212,8 @@
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr"/>
+      <c r="I63" s="4" t="inlineStr"/>
+      <c r="J63" s="4" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
@@ -3121,6 +3257,8 @@
         </is>
       </c>
       <c r="H64" s="5" t="inlineStr"/>
+      <c r="I64" s="5" t="inlineStr"/>
+      <c r="J64" s="5" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -3163,6 +3301,8 @@
         </is>
       </c>
       <c r="H65" s="4" t="inlineStr"/>
+      <c r="I65" s="4" t="inlineStr"/>
+      <c r="J65" s="4" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
@@ -3206,6 +3346,8 @@
         </is>
       </c>
       <c r="H66" s="5" t="inlineStr"/>
+      <c r="I66" s="5" t="inlineStr"/>
+      <c r="J66" s="5" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -3247,6 +3389,8 @@
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr"/>
+      <c r="I67" s="4" t="inlineStr"/>
+      <c r="J67" s="4" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
@@ -3289,6 +3433,8 @@
         </is>
       </c>
       <c r="H68" s="5" t="inlineStr"/>
+      <c r="I68" s="5" t="inlineStr"/>
+      <c r="J68" s="5" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -3331,6 +3477,8 @@
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr"/>
+      <c r="I69" s="4" t="inlineStr"/>
+      <c r="J69" s="4" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
@@ -3373,6 +3521,8 @@
         </is>
       </c>
       <c r="H70" s="5" t="inlineStr"/>
+      <c r="I70" s="5" t="inlineStr"/>
+      <c r="J70" s="5" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -3414,6 +3564,8 @@
         </is>
       </c>
       <c r="H71" s="4" t="inlineStr"/>
+      <c r="I71" s="4" t="inlineStr"/>
+      <c r="J71" s="4" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
@@ -3451,6 +3603,8 @@
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr"/>
+      <c r="I72" s="5" t="inlineStr"/>
+      <c r="J72" s="5" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -3494,6 +3648,8 @@
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr"/>
+      <c r="I73" s="4" t="inlineStr"/>
+      <c r="J73" s="4" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
@@ -3537,6 +3693,8 @@
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr"/>
+      <c r="I74" s="5" t="inlineStr"/>
+      <c r="J74" s="5" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
@@ -3579,6 +3737,8 @@
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr"/>
+      <c r="I75" s="4" t="inlineStr"/>
+      <c r="J75" s="4" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
@@ -3620,6 +3780,8 @@
         </is>
       </c>
       <c r="H76" s="5" t="inlineStr"/>
+      <c r="I76" s="5" t="inlineStr"/>
+      <c r="J76" s="5" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -3663,6 +3825,8 @@
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr"/>
+      <c r="I77" s="4" t="inlineStr"/>
+      <c r="J77" s="4" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
@@ -3706,6 +3870,8 @@
         </is>
       </c>
       <c r="H78" s="5" t="inlineStr"/>
+      <c r="I78" s="5" t="inlineStr"/>
+      <c r="J78" s="5" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -3747,6 +3913,8 @@
         </is>
       </c>
       <c r="H79" s="4" t="inlineStr"/>
+      <c r="I79" s="4" t="inlineStr"/>
+      <c r="J79" s="4" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
@@ -3790,6 +3958,8 @@
         </is>
       </c>
       <c r="H80" s="5" t="inlineStr"/>
+      <c r="I80" s="5" t="inlineStr"/>
+      <c r="J80" s="5" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -3832,6 +4002,8 @@
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr"/>
+      <c r="I81" s="4" t="inlineStr"/>
+      <c r="J81" s="4" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
@@ -3873,6 +4045,8 @@
         </is>
       </c>
       <c r="H82" s="5" t="inlineStr"/>
+      <c r="I82" s="5" t="inlineStr"/>
+      <c r="J82" s="5" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -3914,6 +4088,8 @@
         </is>
       </c>
       <c r="H83" s="4" t="inlineStr"/>
+      <c r="I83" s="4" t="inlineStr"/>
+      <c r="J83" s="4" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
@@ -3956,6 +4132,8 @@
         </is>
       </c>
       <c r="H84" s="5" t="inlineStr"/>
+      <c r="I84" s="5" t="inlineStr"/>
+      <c r="J84" s="5" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -3998,6 +4176,8 @@
         </is>
       </c>
       <c r="H85" s="4" t="inlineStr"/>
+      <c r="I85" s="4" t="inlineStr"/>
+      <c r="J85" s="4" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
@@ -4040,6 +4220,8 @@
         </is>
       </c>
       <c r="H86" s="5" t="inlineStr"/>
+      <c r="I86" s="5" t="inlineStr"/>
+      <c r="J86" s="5" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -4082,6 +4264,8 @@
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr"/>
+      <c r="I87" s="4" t="inlineStr"/>
+      <c r="J87" s="4" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
@@ -4125,6 +4309,8 @@
         </is>
       </c>
       <c r="H88" s="5" t="inlineStr"/>
+      <c r="I88" s="5" t="inlineStr"/>
+      <c r="J88" s="5" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -4166,6 +4352,8 @@
         </is>
       </c>
       <c r="H89" s="4" t="inlineStr"/>
+      <c r="I89" s="4" t="inlineStr"/>
+      <c r="J89" s="4" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
@@ -4208,6 +4396,8 @@
         </is>
       </c>
       <c r="H90" s="5" t="inlineStr"/>
+      <c r="I90" s="5" t="inlineStr"/>
+      <c r="J90" s="5" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
@@ -4252,6 +4442,8 @@
         </is>
       </c>
       <c r="H91" s="4" t="inlineStr"/>
+      <c r="I91" s="4" t="inlineStr"/>
+      <c r="J91" s="4" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
@@ -4295,6 +4487,8 @@
         </is>
       </c>
       <c r="H92" s="5" t="inlineStr"/>
+      <c r="I92" s="5" t="inlineStr"/>
+      <c r="J92" s="5" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -4337,6 +4531,8 @@
         </is>
       </c>
       <c r="H93" s="4" t="inlineStr"/>
+      <c r="I93" s="4" t="inlineStr"/>
+      <c r="J93" s="4" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
@@ -4374,6 +4570,8 @@
         </is>
       </c>
       <c r="H94" s="5" t="inlineStr"/>
+      <c r="I94" s="5" t="inlineStr"/>
+      <c r="J94" s="5" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
@@ -4417,6 +4615,8 @@
         </is>
       </c>
       <c r="H95" s="4" t="inlineStr"/>
+      <c r="I95" s="4" t="inlineStr"/>
+      <c r="J95" s="4" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
@@ -4460,6 +4660,8 @@
         </is>
       </c>
       <c r="H96" s="5" t="inlineStr"/>
+      <c r="I96" s="5" t="inlineStr"/>
+      <c r="J96" s="5" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -4502,6 +4704,8 @@
         </is>
       </c>
       <c r="H97" s="4" t="inlineStr"/>
+      <c r="I97" s="4" t="inlineStr"/>
+      <c r="J97" s="4" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
@@ -4544,6 +4748,8 @@
         </is>
       </c>
       <c r="H98" s="5" t="inlineStr"/>
+      <c r="I98" s="5" t="inlineStr"/>
+      <c r="J98" s="5" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -4585,6 +4791,8 @@
         </is>
       </c>
       <c r="H99" s="4" t="inlineStr"/>
+      <c r="I99" s="4" t="inlineStr"/>
+      <c r="J99" s="4" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
@@ -4626,6 +4834,8 @@
         </is>
       </c>
       <c r="H100" s="5" t="inlineStr"/>
+      <c r="I100" s="5" t="inlineStr"/>
+      <c r="J100" s="5" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -4668,6 +4878,8 @@
         </is>
       </c>
       <c r="H101" s="4" t="inlineStr"/>
+      <c r="I101" s="4" t="inlineStr"/>
+      <c r="J101" s="4" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
@@ -4710,6 +4922,8 @@
         </is>
       </c>
       <c r="H102" s="5" t="inlineStr"/>
+      <c r="I102" s="5" t="inlineStr"/>
+      <c r="J102" s="5" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -4751,6 +4965,8 @@
         </is>
       </c>
       <c r="H103" s="4" t="inlineStr"/>
+      <c r="I103" s="4" t="inlineStr"/>
+      <c r="J103" s="4" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
@@ -4788,6 +5004,8 @@
         </is>
       </c>
       <c r="H104" s="5" t="inlineStr"/>
+      <c r="I104" s="5" t="inlineStr"/>
+      <c r="J104" s="5" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -4829,6 +5047,8 @@
         </is>
       </c>
       <c r="H105" s="4" t="inlineStr"/>
+      <c r="I105" s="4" t="inlineStr"/>
+      <c r="J105" s="4" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
@@ -4871,6 +5091,8 @@
         </is>
       </c>
       <c r="H106" s="5" t="inlineStr"/>
+      <c r="I106" s="5" t="inlineStr"/>
+      <c r="J106" s="5" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
@@ -4914,6 +5136,8 @@
         </is>
       </c>
       <c r="H107" s="4" t="inlineStr"/>
+      <c r="I107" s="4" t="inlineStr"/>
+      <c r="J107" s="4" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
@@ -4956,6 +5180,8 @@
         </is>
       </c>
       <c r="H108" s="5" t="inlineStr"/>
+      <c r="I108" s="5" t="inlineStr"/>
+      <c r="J108" s="5" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -4990,6 +5216,8 @@
       </c>
       <c r="G109" s="4" t="inlineStr"/>
       <c r="H109" s="4" t="inlineStr"/>
+      <c r="I109" s="4" t="inlineStr"/>
+      <c r="J109" s="4" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
@@ -5031,6 +5259,8 @@
         </is>
       </c>
       <c r="H110" s="5" t="inlineStr"/>
+      <c r="I110" s="5" t="inlineStr"/>
+      <c r="J110" s="5" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
@@ -5071,6 +5301,8 @@
         </is>
       </c>
       <c r="H111" s="4" t="inlineStr"/>
+      <c r="I111" s="4" t="inlineStr"/>
+      <c r="J111" s="4" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
@@ -5112,6 +5344,8 @@
         </is>
       </c>
       <c r="H112" s="5" t="inlineStr"/>
+      <c r="I112" s="5" t="inlineStr"/>
+      <c r="J112" s="5" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
@@ -5155,6 +5389,8 @@
         </is>
       </c>
       <c r="H113" s="4" t="inlineStr"/>
+      <c r="I113" s="4" t="inlineStr"/>
+      <c r="J113" s="4" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="5" t="inlineStr">
@@ -5197,6 +5433,8 @@
         </is>
       </c>
       <c r="H114" s="5" t="inlineStr"/>
+      <c r="I114" s="5" t="inlineStr"/>
+      <c r="J114" s="5" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
@@ -5239,6 +5477,8 @@
         </is>
       </c>
       <c r="H115" s="4" t="inlineStr"/>
+      <c r="I115" s="4" t="inlineStr"/>
+      <c r="J115" s="4" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
@@ -5281,6 +5521,8 @@
         </is>
       </c>
       <c r="H116" s="5" t="inlineStr"/>
+      <c r="I116" s="5" t="inlineStr"/>
+      <c r="J116" s="5" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
@@ -5323,6 +5565,8 @@
         </is>
       </c>
       <c r="H117" s="4" t="inlineStr"/>
+      <c r="I117" s="4" t="inlineStr"/>
+      <c r="J117" s="4" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
@@ -5364,6 +5608,8 @@
         </is>
       </c>
       <c r="H118" s="5" t="inlineStr"/>
+      <c r="I118" s="5" t="inlineStr"/>
+      <c r="J118" s="5" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
@@ -5406,6 +5652,8 @@
         </is>
       </c>
       <c r="H119" s="4" t="inlineStr"/>
+      <c r="I119" s="4" t="inlineStr"/>
+      <c r="J119" s="4" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
@@ -5453,6 +5701,8 @@
         </is>
       </c>
       <c r="H120" s="5" t="inlineStr"/>
+      <c r="I120" s="5" t="inlineStr"/>
+      <c r="J120" s="5" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
@@ -5495,6 +5745,8 @@
         </is>
       </c>
       <c r="H121" s="4" t="inlineStr"/>
+      <c r="I121" s="4" t="inlineStr"/>
+      <c r="J121" s="4" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
@@ -5537,6 +5789,8 @@
         </is>
       </c>
       <c r="H122" s="5" t="inlineStr"/>
+      <c r="I122" s="5" t="inlineStr"/>
+      <c r="J122" s="5" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
@@ -5577,6 +5831,8 @@
       </c>
       <c r="G123" s="4" t="inlineStr"/>
       <c r="H123" s="4" t="inlineStr"/>
+      <c r="I123" s="4" t="inlineStr"/>
+      <c r="J123" s="4" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
@@ -5613,6 +5869,8 @@
       </c>
       <c r="G124" s="5" t="inlineStr"/>
       <c r="H124" s="5" t="inlineStr"/>
+      <c r="I124" s="5" t="inlineStr"/>
+      <c r="J124" s="5" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
@@ -5654,6 +5912,8 @@
         </is>
       </c>
       <c r="H125" s="4" t="inlineStr"/>
+      <c r="I125" s="4" t="inlineStr"/>
+      <c r="J125" s="4" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="5" t="inlineStr">
@@ -5683,6 +5943,8 @@
       <c r="F126" s="5" t="inlineStr"/>
       <c r="G126" s="5" t="inlineStr"/>
       <c r="H126" s="5" t="inlineStr"/>
+      <c r="I126" s="5" t="inlineStr"/>
+      <c r="J126" s="5" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
@@ -5725,6 +5987,8 @@
         </is>
       </c>
       <c r="H127" s="4" t="inlineStr"/>
+      <c r="I127" s="4" t="inlineStr"/>
+      <c r="J127" s="4" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
@@ -5766,6 +6030,8 @@
         </is>
       </c>
       <c r="H128" s="5" t="inlineStr"/>
+      <c r="I128" s="5" t="inlineStr"/>
+      <c r="J128" s="5" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
@@ -5806,6 +6072,8 @@
       </c>
       <c r="G129" s="4" t="inlineStr"/>
       <c r="H129" s="4" t="inlineStr"/>
+      <c r="I129" s="4" t="inlineStr"/>
+      <c r="J129" s="4" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="5" t="inlineStr">
@@ -5843,6 +6111,8 @@
       </c>
       <c r="G130" s="5" t="inlineStr"/>
       <c r="H130" s="5" t="inlineStr"/>
+      <c r="I130" s="5" t="inlineStr"/>
+      <c r="J130" s="5" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
@@ -5884,6 +6154,8 @@
         </is>
       </c>
       <c r="H131" s="4" t="inlineStr"/>
+      <c r="I131" s="4" t="inlineStr"/>
+      <c r="J131" s="4" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="5" t="inlineStr">
@@ -5929,6 +6201,8 @@
         </is>
       </c>
       <c r="H132" s="5" t="inlineStr"/>
+      <c r="I132" s="5" t="inlineStr"/>
+      <c r="J132" s="5" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
@@ -5974,6 +6248,8 @@
         </is>
       </c>
       <c r="H133" s="4" t="inlineStr"/>
+      <c r="I133" s="4" t="inlineStr"/>
+      <c r="J133" s="4" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="5" t="inlineStr">
@@ -6015,6 +6291,8 @@
         </is>
       </c>
       <c r="H134" s="5" t="inlineStr"/>
+      <c r="I134" s="5" t="inlineStr"/>
+      <c r="J134" s="5" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
@@ -6055,6 +6333,8 @@
       </c>
       <c r="G135" s="4" t="inlineStr"/>
       <c r="H135" s="4" t="inlineStr"/>
+      <c r="I135" s="4" t="inlineStr"/>
+      <c r="J135" s="4" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="5" t="inlineStr">
@@ -6097,6 +6377,8 @@
         </is>
       </c>
       <c r="H136" s="5" t="inlineStr"/>
+      <c r="I136" s="5" t="inlineStr"/>
+      <c r="J136" s="5" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
@@ -6140,6 +6422,8 @@
         </is>
       </c>
       <c r="H137" s="4" t="inlineStr"/>
+      <c r="I137" s="4" t="inlineStr"/>
+      <c r="J137" s="4" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="5" t="inlineStr">
@@ -6183,6 +6467,8 @@
         </is>
       </c>
       <c r="H138" s="5" t="inlineStr"/>
+      <c r="I138" s="5" t="inlineStr"/>
+      <c r="J138" s="5" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
@@ -6224,6 +6510,8 @@
       </c>
       <c r="G139" s="4" t="inlineStr"/>
       <c r="H139" s="4" t="inlineStr"/>
+      <c r="I139" s="4" t="inlineStr"/>
+      <c r="J139" s="4" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="5" t="inlineStr">
@@ -6262,6 +6550,8 @@
       </c>
       <c r="G140" s="5" t="inlineStr"/>
       <c r="H140" s="5" t="inlineStr"/>
+      <c r="I140" s="5" t="inlineStr"/>
+      <c r="J140" s="5" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -6306,6 +6596,8 @@
         </is>
       </c>
       <c r="H141" s="4" t="inlineStr"/>
+      <c r="I141" s="4" t="inlineStr"/>
+      <c r="J141" s="4" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="5" t="inlineStr">
@@ -6349,6 +6641,8 @@
         </is>
       </c>
       <c r="H142" s="5" t="inlineStr"/>
+      <c r="I142" s="5" t="inlineStr"/>
+      <c r="J142" s="5" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
@@ -6391,6 +6685,8 @@
         </is>
       </c>
       <c r="H143" s="4" t="inlineStr"/>
+      <c r="I143" s="4" t="inlineStr"/>
+      <c r="J143" s="4" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="5" t="inlineStr">
@@ -6429,6 +6725,8 @@
       </c>
       <c r="G144" s="5" t="inlineStr"/>
       <c r="H144" s="5" t="inlineStr"/>
+      <c r="I144" s="5" t="inlineStr"/>
+      <c r="J144" s="5" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
@@ -6469,6 +6767,8 @@
       </c>
       <c r="G145" s="4" t="inlineStr"/>
       <c r="H145" s="4" t="inlineStr"/>
+      <c r="I145" s="4" t="inlineStr"/>
+      <c r="J145" s="4" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="5" t="inlineStr">
@@ -6510,6 +6810,8 @@
       </c>
       <c r="G146" s="5" t="inlineStr"/>
       <c r="H146" s="5" t="inlineStr"/>
+      <c r="I146" s="5" t="inlineStr"/>
+      <c r="J146" s="5" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
@@ -6549,6 +6851,8 @@
       </c>
       <c r="G147" s="4" t="inlineStr"/>
       <c r="H147" s="4" t="inlineStr"/>
+      <c r="I147" s="4" t="inlineStr"/>
+      <c r="J147" s="4" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="5" t="inlineStr">
@@ -6598,6 +6902,8 @@
       </c>
       <c r="G148" s="5" t="inlineStr"/>
       <c r="H148" s="5" t="inlineStr"/>
+      <c r="I148" s="5" t="inlineStr"/>
+      <c r="J148" s="5" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
@@ -6656,6 +6962,8 @@
         </is>
       </c>
       <c r="H149" s="4" t="inlineStr"/>
+      <c r="I149" s="4" t="inlineStr"/>
+      <c r="J149" s="4" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="5" t="inlineStr">
@@ -6705,6 +7013,8 @@
         </is>
       </c>
       <c r="H150" s="5" t="inlineStr"/>
+      <c r="I150" s="5" t="inlineStr"/>
+      <c r="J150" s="5" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
@@ -6753,6 +7063,8 @@
       </c>
       <c r="G151" s="4" t="inlineStr"/>
       <c r="H151" s="4" t="inlineStr"/>
+      <c r="I151" s="4" t="inlineStr"/>
+      <c r="J151" s="4" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="5" t="inlineStr">
@@ -6798,6 +7110,8 @@
         </is>
       </c>
       <c r="H152" s="5" t="inlineStr"/>
+      <c r="I152" s="5" t="inlineStr"/>
+      <c r="J152" s="5" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
@@ -6840,6 +7154,8 @@
         </is>
       </c>
       <c r="H153" s="4" t="inlineStr"/>
+      <c r="I153" s="4" t="inlineStr"/>
+      <c r="J153" s="4" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="5" t="inlineStr">
@@ -6883,6 +7199,8 @@
         </is>
       </c>
       <c r="H154" s="5" t="inlineStr"/>
+      <c r="I154" s="5" t="inlineStr"/>
+      <c r="J154" s="5" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
@@ -6925,6 +7243,8 @@
         </is>
       </c>
       <c r="H155" s="4" t="inlineStr"/>
+      <c r="I155" s="4" t="inlineStr"/>
+      <c r="J155" s="4" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="5" t="inlineStr">
@@ -6984,6 +7304,8 @@
         </is>
       </c>
       <c r="H156" s="5" t="inlineStr"/>
+      <c r="I156" s="5" t="inlineStr"/>
+      <c r="J156" s="5" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
@@ -7028,6 +7350,8 @@
       </c>
       <c r="G157" s="4" t="inlineStr"/>
       <c r="H157" s="4" t="inlineStr"/>
+      <c r="I157" s="4" t="inlineStr"/>
+      <c r="J157" s="4" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="5" t="inlineStr">
@@ -7076,6 +7400,8 @@
       </c>
       <c r="G158" s="5" t="inlineStr"/>
       <c r="H158" s="5" t="inlineStr"/>
+      <c r="I158" s="5" t="inlineStr"/>
+      <c r="J158" s="5" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
@@ -7127,6 +7453,8 @@
         </is>
       </c>
       <c r="H159" s="4" t="inlineStr"/>
+      <c r="I159" s="4" t="inlineStr"/>
+      <c r="J159" s="4" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="5" t="inlineStr">
@@ -7168,6 +7496,8 @@
       </c>
       <c r="G160" s="5" t="inlineStr"/>
       <c r="H160" s="5" t="inlineStr"/>
+      <c r="I160" s="5" t="inlineStr"/>
+      <c r="J160" s="5" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
@@ -7213,6 +7543,8 @@
         </is>
       </c>
       <c r="H161" s="4" t="inlineStr"/>
+      <c r="I161" s="4" t="inlineStr"/>
+      <c r="J161" s="4" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="5" t="inlineStr">
@@ -7266,6 +7598,8 @@
         </is>
       </c>
       <c r="H162" s="5" t="inlineStr"/>
+      <c r="I162" s="5" t="inlineStr"/>
+      <c r="J162" s="5" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
@@ -7312,6 +7646,8 @@
         </is>
       </c>
       <c r="H163" s="4" t="inlineStr"/>
+      <c r="I163" s="4" t="inlineStr"/>
+      <c r="J163" s="4" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="5" t="inlineStr">
@@ -7352,6 +7688,8 @@
       </c>
       <c r="G164" s="5" t="inlineStr"/>
       <c r="H164" s="5" t="inlineStr"/>
+      <c r="I164" s="5" t="inlineStr"/>
+      <c r="J164" s="5" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
@@ -7393,6 +7731,8 @@
       </c>
       <c r="G165" s="4" t="inlineStr"/>
       <c r="H165" s="4" t="inlineStr"/>
+      <c r="I165" s="4" t="inlineStr"/>
+      <c r="J165" s="4" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="5" t="inlineStr">
@@ -7428,6 +7768,8 @@
       </c>
       <c r="G166" s="5" t="inlineStr"/>
       <c r="H166" s="5" t="inlineStr"/>
+      <c r="I166" s="5" t="inlineStr"/>
+      <c r="J166" s="5" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
@@ -7471,6 +7813,8 @@
       </c>
       <c r="G167" s="4" t="inlineStr"/>
       <c r="H167" s="4" t="inlineStr"/>
+      <c r="I167" s="4" t="inlineStr"/>
+      <c r="J167" s="4" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="5" t="inlineStr">
@@ -7506,6 +7850,8 @@
       </c>
       <c r="G168" s="5" t="inlineStr"/>
       <c r="H168" s="5" t="inlineStr"/>
+      <c r="I168" s="5" t="inlineStr"/>
+      <c r="J168" s="5" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
@@ -7545,6 +7891,8 @@
       </c>
       <c r="G169" s="4" t="inlineStr"/>
       <c r="H169" s="4" t="inlineStr"/>
+      <c r="I169" s="4" t="inlineStr"/>
+      <c r="J169" s="4" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="5" t="inlineStr">
@@ -7594,6 +7942,8 @@
       </c>
       <c r="G170" s="5" t="inlineStr"/>
       <c r="H170" s="5" t="inlineStr"/>
+      <c r="I170" s="5" t="inlineStr"/>
+      <c r="J170" s="5" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
@@ -7637,6 +7987,8 @@
       </c>
       <c r="G171" s="4" t="inlineStr"/>
       <c r="H171" s="4" t="inlineStr"/>
+      <c r="I171" s="4" t="inlineStr"/>
+      <c r="J171" s="4" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="5" t="inlineStr">
@@ -7674,6 +8026,8 @@
       </c>
       <c r="G172" s="5" t="inlineStr"/>
       <c r="H172" s="5" t="inlineStr"/>
+      <c r="I172" s="5" t="inlineStr"/>
+      <c r="J172" s="5" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
@@ -7711,6 +8065,8 @@
       </c>
       <c r="G173" s="4" t="inlineStr"/>
       <c r="H173" s="4" t="inlineStr"/>
+      <c r="I173" s="4" t="inlineStr"/>
+      <c r="J173" s="4" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="5" t="inlineStr">
@@ -7751,6 +8107,8 @@
       </c>
       <c r="G174" s="5" t="inlineStr"/>
       <c r="H174" s="5" t="inlineStr"/>
+      <c r="I174" s="5" t="inlineStr"/>
+      <c r="J174" s="5" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
@@ -7788,6 +8146,8 @@
       </c>
       <c r="G175" s="4" t="inlineStr"/>
       <c r="H175" s="4" t="inlineStr"/>
+      <c r="I175" s="4" t="inlineStr"/>
+      <c r="J175" s="4" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="5" t="inlineStr">
@@ -7833,6 +8193,8 @@
       </c>
       <c r="G176" s="5" t="inlineStr"/>
       <c r="H176" s="5" t="inlineStr"/>
+      <c r="I176" s="5" t="inlineStr"/>
+      <c r="J176" s="5" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
@@ -7874,6 +8236,8 @@
       </c>
       <c r="G177" s="4" t="inlineStr"/>
       <c r="H177" s="4" t="inlineStr"/>
+      <c r="I177" s="4" t="inlineStr"/>
+      <c r="J177" s="4" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="5" t="inlineStr">
@@ -7914,6 +8278,8 @@
       </c>
       <c r="G178" s="5" t="inlineStr"/>
       <c r="H178" s="5" t="inlineStr"/>
+      <c r="I178" s="5" t="inlineStr"/>
+      <c r="J178" s="5" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
@@ -7953,6 +8319,8 @@
       </c>
       <c r="G179" s="4" t="inlineStr"/>
       <c r="H179" s="4" t="inlineStr"/>
+      <c r="I179" s="4" t="inlineStr"/>
+      <c r="J179" s="4" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="5" t="inlineStr">
@@ -7994,6 +8362,8 @@
       </c>
       <c r="G180" s="5" t="inlineStr"/>
       <c r="H180" s="5" t="inlineStr"/>
+      <c r="I180" s="5" t="inlineStr"/>
+      <c r="J180" s="5" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
@@ -8027,6 +8397,8 @@
       </c>
       <c r="G181" s="4" t="inlineStr"/>
       <c r="H181" s="4" t="inlineStr"/>
+      <c r="I181" s="4" t="inlineStr"/>
+      <c r="J181" s="4" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="5" t="inlineStr">
@@ -8067,6 +8439,8 @@
       </c>
       <c r="G182" s="5" t="inlineStr"/>
       <c r="H182" s="5" t="inlineStr"/>
+      <c r="I182" s="5" t="inlineStr"/>
+      <c r="J182" s="5" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
@@ -8104,6 +8478,8 @@
       </c>
       <c r="G183" s="4" t="inlineStr"/>
       <c r="H183" s="4" t="inlineStr"/>
+      <c r="I183" s="4" t="inlineStr"/>
+      <c r="J183" s="4" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="5" t="inlineStr">
@@ -8142,6 +8518,8 @@
       </c>
       <c r="G184" s="5" t="inlineStr"/>
       <c r="H184" s="5" t="inlineStr"/>
+      <c r="I184" s="5" t="inlineStr"/>
+      <c r="J184" s="5" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
@@ -8202,6 +8580,8 @@
       </c>
       <c r="G185" s="4" t="inlineStr"/>
       <c r="H185" s="4" t="inlineStr"/>
+      <c r="I185" s="4" t="inlineStr"/>
+      <c r="J185" s="4" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="5" t="inlineStr">
@@ -8238,6 +8618,8 @@
       </c>
       <c r="G186" s="5" t="inlineStr"/>
       <c r="H186" s="5" t="inlineStr"/>
+      <c r="I186" s="5" t="inlineStr"/>
+      <c r="J186" s="5" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
@@ -8271,6 +8653,8 @@
       </c>
       <c r="G187" s="4" t="inlineStr"/>
       <c r="H187" s="4" t="inlineStr"/>
+      <c r="I187" s="4" t="inlineStr"/>
+      <c r="J187" s="4" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="5" t="inlineStr">
@@ -8311,6 +8695,8 @@
       </c>
       <c r="G188" s="5" t="inlineStr"/>
       <c r="H188" s="5" t="inlineStr"/>
+      <c r="I188" s="5" t="inlineStr"/>
+      <c r="J188" s="5" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
@@ -8346,6 +8732,8 @@
       </c>
       <c r="G189" s="4" t="inlineStr"/>
       <c r="H189" s="4" t="inlineStr"/>
+      <c r="I189" s="4" t="inlineStr"/>
+      <c r="J189" s="4" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="5" t="inlineStr">
@@ -8391,6 +8779,8 @@
       </c>
       <c r="G190" s="5" t="inlineStr"/>
       <c r="H190" s="5" t="inlineStr"/>
+      <c r="I190" s="5" t="inlineStr"/>
+      <c r="J190" s="5" t="inlineStr"/>
     </row>
     <row r="191" ht="25" customHeight="1">
       <c r="A191" s="2" t="inlineStr">
@@ -8405,6 +8795,8 @@
       <c r="F191" s="3" t="n"/>
       <c r="G191" s="3" t="n"/>
       <c r="H191" s="3" t="n"/>
+      <c r="I191" s="3" t="n"/>
+      <c r="J191" s="3" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="6" t="inlineStr">
@@ -8450,12 +8842,14 @@
       <c r="F192" s="6" t="inlineStr"/>
       <c r="G192" s="6" t="inlineStr"/>
       <c r="H192" s="6" t="inlineStr"/>
+      <c r="I192" s="6" t="inlineStr"/>
+      <c r="J192" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H192"/>
+  <autoFilter ref="A1:J192"/>
   <mergeCells count="2">
-    <mergeCell ref="A191:H191"/>
-    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A191:J191"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>